<commit_message>
Legg til prismodell for T. Solbakken Trafikkskole
Linje 80: kr 1500/mnd fast (telefonkanal + tilgjengelighet, ingen
samtaler inkludert) + kr 950 per påbegynt 20-samtalersteg besvarte
samtaler (1-20=1x950, 21-40=2x950, osv). Bekreftet av Geir
2026-09-15. Med augusttallene (H=59, dvs. tredje 20-steg) blir
beregnet pris 1500+3*950 = 4350 kr.

Utvidet BEREGNET TOTAL / FAKTISK TOTAL til å telle med linje 79-80
(bruker to separate SUM-ranges, I4:I95 + I99:I101, for å unngå at
totalradene summerer seg selv). Kinnarps (linje 79) er fortsatt uten
prismodell og teller 0 i totalen inntil videre.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QPGt8PSp7APbNpsmbE3wCA
</commit_message>
<xml_diff>
--- a/data/PrisoversiktSentralbord2026.xlsx
+++ b/data/PrisoversiktSentralbord2026.xlsx
@@ -74,7 +74,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="811" uniqueCount="462">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="814" uniqueCount="465">
   <si>
     <t xml:space="preserve">We4you AS – Prisoversikt Sentralbord 2026  |  Augusr2026  |  Beregnet vs Faktisk (Tripletex)</t>
   </si>
@@ -842,7 +842,16 @@
     <t xml:space="preserve">T. Solbakken Trafikkskole</t>
   </si>
   <si>
-    <t xml:space="preserve">Ny kø funnet i Zisson august 2026 (2963) – prismodell ikke avtalt ennå</t>
+    <t xml:space="preserve">Fast pris + trappepris per 20 besvarte samtaler</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kr 1 500 / mnd fast + kr 950 per påbegynt 20-samtalersteg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ingen samtaler inkl. i fastprisen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fast kr 1500/mnd (telefonkanal + tilgjengelighet). + kr 950 per påbegynt 20-steg besvarte samtaler (1-20=1x950, 21-40=2x950, 41-60=3x950, osv). Prismodell bekreftet av Geir 2026-09-15.</t>
   </si>
   <si>
     <t xml:space="preserve">Vol fra</t>
@@ -5508,8 +5517,8 @@
       <c r="H96" s="55"/>
       <c r="I96" s="55"/>
       <c r="J96" s="56" t="n">
-        <f aca="false">SUM(I4:I93)</f>
-        <v>281139</v>
+        <f aca="false">SUM(I4:I95,I99:I101)</f>
+        <v>285489</v>
       </c>
     </row>
     <row r="97" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5525,12 +5534,12 @@
       <c r="H97" s="55"/>
       <c r="I97" s="55"/>
       <c r="J97" s="56" t="n">
-        <f aca="false">SUM(J4:J93)</f>
+        <f aca="false">SUM(J4:J95,J99:J101)</f>
         <v>278757</v>
       </c>
       <c r="K97" s="57" t="n">
         <f aca="false">J97-J96</f>
-        <v>-2382</v>
+        <v>-6732</v>
       </c>
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5563,13 +5572,26 @@
         <v>253</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>251</v>
+        <v>14</v>
+      </c>
+      <c r="D101" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>256</v>
       </c>
       <c r="G101" s="1" t="s">
-        <v>254</v>
+        <v>257</v>
       </c>
       <c r="H101" s="1" t="n">
         <v>59</v>
+      </c>
+      <c r="I101" s="1" t="n">
+        <f aca="false">IF(H101="–","–",1500+ROUNDUP(H101/20,0)*950)</f>
+        <v>4350</v>
       </c>
     </row>
   </sheetData>
@@ -5608,7 +5630,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="79" t="s">
-        <v>414</v>
+        <v>417</v>
       </c>
       <c r="B2" s="70"/>
       <c r="C2" s="70"/>
@@ -5631,61 +5653,61 @@
         <v>2</v>
       </c>
       <c r="B4" s="69" t="s">
-        <v>415</v>
+        <v>418</v>
       </c>
       <c r="D4" s="69" t="s">
-        <v>416</v>
+        <v>419</v>
       </c>
       <c r="E4" s="69" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="F4" s="69" t="s">
-        <v>418</v>
+        <v>421</v>
       </c>
       <c r="G4" s="69" t="s">
-        <v>419</v>
+        <v>422</v>
       </c>
       <c r="I4" s="80" t="s">
-        <v>420</v>
+        <v>423</v>
       </c>
       <c r="J4" s="81" t="s">
-        <v>421</v>
+        <v>424</v>
       </c>
       <c r="K4" s="82" t="s">
-        <v>422</v>
+        <v>425</v>
       </c>
       <c r="L4" s="80" t="s">
-        <v>423</v>
+        <v>426</v>
       </c>
       <c r="M4" s="81" t="s">
-        <v>424</v>
+        <v>427</v>
       </c>
       <c r="N4" s="82" t="s">
-        <v>425</v>
+        <v>428</v>
       </c>
       <c r="O4" s="80" t="s">
-        <v>426</v>
+        <v>429</v>
       </c>
       <c r="P4" s="81" t="s">
-        <v>427</v>
+        <v>430</v>
       </c>
       <c r="Q4" s="82" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="R4" s="80" t="s">
-        <v>429</v>
+        <v>432</v>
       </c>
       <c r="S4" s="81" t="s">
-        <v>430</v>
+        <v>433</v>
       </c>
       <c r="T4" s="82" t="s">
-        <v>431</v>
+        <v>434</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="70"/>
       <c r="B5" s="69" t="s">
-        <v>432</v>
+        <v>435</v>
       </c>
       <c r="D5" s="70"/>
       <c r="E5" s="70"/>
@@ -5746,38 +5768,38 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="73" t="s">
-        <v>433</v>
+        <v>436</v>
       </c>
       <c r="B8" s="70" t="n">
         <v>32693</v>
       </c>
       <c r="D8" s="70" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="E8" s="70"/>
       <c r="F8" s="70" t="s">
-        <v>435</v>
+        <v>438</v>
       </c>
       <c r="G8" s="91" t="s">
-        <v>436</v>
+        <v>439</v>
       </c>
       <c r="I8" s="83" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="J8" s="84"/>
       <c r="K8" s="85"/>
       <c r="L8" s="83" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="M8" s="84"/>
       <c r="N8" s="85"/>
       <c r="O8" s="83" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="P8" s="84"/>
       <c r="Q8" s="85"/>
       <c r="R8" s="86" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="S8" s="90"/>
       <c r="T8" s="88"/>
@@ -5804,40 +5826,40 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="73" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="B10" s="70" t="n">
         <v>32710</v>
       </c>
       <c r="D10" s="70" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="E10" s="70"/>
       <c r="F10" s="70" t="s">
+        <v>442</v>
+      </c>
+      <c r="G10" s="91" t="s">
         <v>439</v>
-      </c>
-      <c r="G10" s="91" t="s">
-        <v>436</v>
       </c>
       <c r="I10" s="83"/>
       <c r="J10" s="84"/>
       <c r="K10" s="85" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="L10" s="83"/>
       <c r="M10" s="84"/>
       <c r="N10" s="85" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="O10" s="83"/>
       <c r="P10" s="84"/>
       <c r="Q10" s="85" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="R10" s="86"/>
       <c r="S10" s="90"/>
       <c r="T10" s="88" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5863,50 +5885,50 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="93" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="B12" s="70" t="n">
         <v>30308</v>
       </c>
       <c r="C12" s="70" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="D12" s="70" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="E12" s="70" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="F12" s="70" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="G12" s="89" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="I12" s="83"/>
       <c r="J12" s="84" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="K12" s="85"/>
       <c r="L12" s="83"/>
       <c r="M12" s="84" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="N12" s="85"/>
       <c r="O12" s="83"/>
       <c r="P12" s="84" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="Q12" s="85"/>
       <c r="R12" s="86"/>
       <c r="S12" s="90" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="T12" s="88"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="72" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="B13" s="70"/>
       <c r="C13" s="70"/>
@@ -5934,42 +5956,42 @@
       <c r="B14" s="70"/>
       <c r="C14" s="70"/>
       <c r="D14" s="70" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="E14" s="70"/>
       <c r="F14" s="70" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="G14" s="89" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="I14" s="83"/>
       <c r="J14" s="84" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="K14" s="85" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="L14" s="83"/>
       <c r="M14" s="84"/>
       <c r="N14" s="85" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="O14" s="83"/>
       <c r="P14" s="84"/>
       <c r="Q14" s="85" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="R14" s="86"/>
       <c r="S14" s="87"/>
       <c r="T14" s="88" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="I15" s="83"/>
       <c r="J15" s="84" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="K15" s="85"/>
       <c r="L15" s="83"/>
@@ -5984,16 +6006,16 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="73" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="D16" s="70" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="F16" s="70" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="G16" s="70" t="s">
-        <v>428</v>
+        <v>431</v>
       </c>
       <c r="I16" s="83"/>
       <c r="J16" s="84"/>
@@ -6003,10 +6025,10 @@
       <c r="N16" s="85"/>
       <c r="O16" s="83"/>
       <c r="P16" s="84" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="Q16" s="85" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="R16" s="86"/>
       <c r="S16" s="90"/>
@@ -6014,11 +6036,11 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="F17" s="70" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="I17" s="83"/>
       <c r="J17" s="84" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="K17" s="85"/>
       <c r="L17" s="83"/>
@@ -6033,39 +6055,39 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="73" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="B18" s="1" t="n">
         <v>33010</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>434</v>
+        <v>437</v>
       </c>
       <c r="F18" s="70" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="I18" s="83" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="J18" s="84" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="K18" s="85"/>
       <c r="L18" s="83" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="M18" s="84"/>
       <c r="N18" s="85"/>
       <c r="O18" s="83" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="P18" s="84"/>
       <c r="Q18" s="85"/>
       <c r="R18" s="86" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="S18" s="87"/>
       <c r="T18" s="88"/>
@@ -6073,7 +6095,7 @@
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="I19" s="83"/>
       <c r="J19" s="84" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="K19" s="85"/>
       <c r="L19" s="83"/>
@@ -6089,7 +6111,7 @@
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="I20" s="83"/>
       <c r="J20" s="84" t="s">
-        <v>417</v>
+        <v>420</v>
       </c>
       <c r="K20" s="85"/>
       <c r="L20" s="83"/>
@@ -6124,40 +6146,40 @@
   <sheetData>
     <row r="1" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6761,16 +6783,16 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="60" t="s">
-        <v>255</v>
+        <v>258</v>
       </c>
       <c r="B2" s="60" t="s">
-        <v>256</v>
+        <v>259</v>
       </c>
       <c r="C2" s="60"/>
       <c r="D2" s="61"/>
       <c r="E2" s="62"/>
       <c r="F2" s="63" t="s">
-        <v>257</v>
+        <v>260</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7545,7 +7567,7 @@
         <v>14</v>
       </c>
       <c r="C31" s="51" t="s">
-        <v>258</v>
+        <v>261</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="140.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7583,25 +7605,25 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="59" t="s">
-        <v>259</v>
+        <v>262</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>263</v>
+        <v>266</v>
       </c>
       <c r="B4" s="56" t="n">
         <v>1500</v>
@@ -7609,7 +7631,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>264</v>
+        <v>267</v>
       </c>
       <c r="B5" s="56" t="n">
         <v>2280</v>
@@ -7617,7 +7639,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>265</v>
+        <v>268</v>
       </c>
       <c r="B6" s="56" t="n">
         <v>2870</v>
@@ -7625,7 +7647,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>266</v>
+        <v>269</v>
       </c>
       <c r="B7" s="56" t="n">
         <v>3260</v>
@@ -7633,7 +7655,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="s">
-        <v>267</v>
+        <v>270</v>
       </c>
       <c r="B8" s="56" t="n">
         <v>3450</v>
@@ -7641,7 +7663,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="s">
-        <v>268</v>
+        <v>271</v>
       </c>
       <c r="B9" s="56" t="n">
         <v>3810</v>
@@ -7649,7 +7671,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="s">
-        <v>269</v>
+        <v>272</v>
       </c>
       <c r="B10" s="56" t="n">
         <v>4020</v>
@@ -7657,7 +7679,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="s">
-        <v>270</v>
+        <v>273</v>
       </c>
       <c r="B11" s="56" t="n">
         <v>4260</v>
@@ -7665,7 +7687,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="s">
-        <v>271</v>
+        <v>274</v>
       </c>
       <c r="B12" s="56" t="n">
         <v>4490</v>
@@ -7673,7 +7695,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="s">
-        <v>272</v>
+        <v>275</v>
       </c>
       <c r="B13" s="56" t="n">
         <v>4860</v>
@@ -7681,7 +7703,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="s">
-        <v>273</v>
+        <v>276</v>
       </c>
       <c r="B14" s="56" t="n">
         <v>5280</v>
@@ -7689,7 +7711,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B15" s="56" t="n">
         <v>5690</v>
@@ -7697,7 +7719,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="B16" s="56" t="n">
         <v>6100</v>
@@ -7705,7 +7727,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="B17" s="56" t="n">
         <v>6520</v>
@@ -7713,7 +7735,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="s">
-        <v>277</v>
+        <v>280</v>
       </c>
       <c r="B18" s="56" t="n">
         <v>6940</v>
@@ -7721,7 +7743,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B19" s="56" t="n">
         <v>7370</v>
@@ -7729,7 +7751,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="B20" s="56" t="n">
         <v>7790</v>
@@ -7737,7 +7759,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="B21" s="56" t="n">
         <v>8200</v>
@@ -7745,7 +7767,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="s">
-        <v>281</v>
+        <v>284</v>
       </c>
       <c r="B22" s="56" t="n">
         <v>8610</v>
@@ -7753,7 +7775,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B23" s="56" t="n">
         <v>9020</v>
@@ -7761,7 +7783,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="s">
-        <v>283</v>
+        <v>286</v>
       </c>
       <c r="B24" s="56" t="n">
         <v>9440</v>
@@ -7769,7 +7791,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="s">
-        <v>284</v>
+        <v>287</v>
       </c>
       <c r="B25" s="56" t="n">
         <v>9860</v>
@@ -7777,7 +7799,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="s">
-        <v>285</v>
+        <v>288</v>
       </c>
       <c r="B26" s="56" t="n">
         <v>10280</v>
@@ -7785,7 +7807,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="s">
-        <v>286</v>
+        <v>289</v>
       </c>
       <c r="B27" s="56" t="n">
         <v>10700</v>
@@ -7793,7 +7815,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="s">
-        <v>287</v>
+        <v>290</v>
       </c>
       <c r="B28" s="56" t="n">
         <v>11120</v>
@@ -7801,7 +7823,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="1" t="s">
-        <v>288</v>
+        <v>291</v>
       </c>
       <c r="B29" s="56" t="n">
         <v>11530</v>
@@ -7809,7 +7831,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="1" t="s">
-        <v>289</v>
+        <v>292</v>
       </c>
       <c r="B30" s="56" t="n">
         <v>11940</v>
@@ -7817,7 +7839,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="1" t="s">
-        <v>290</v>
+        <v>293</v>
       </c>
       <c r="B31" s="56" t="n">
         <v>12350</v>
@@ -7825,7 +7847,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="1" t="s">
-        <v>291</v>
+        <v>294</v>
       </c>
       <c r="B32" s="56" t="n">
         <v>12760</v>
@@ -7833,7 +7855,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="1" t="s">
-        <v>292</v>
+        <v>295</v>
       </c>
       <c r="B33" s="56" t="n">
         <v>13180</v>
@@ -7841,7 +7863,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="1" t="s">
-        <v>293</v>
+        <v>296</v>
       </c>
       <c r="B34" s="56" t="n">
         <v>13610</v>
@@ -7849,7 +7871,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="1" t="s">
-        <v>294</v>
+        <v>297</v>
       </c>
       <c r="B35" s="56" t="n">
         <v>14030</v>
@@ -7857,7 +7879,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="1" t="s">
-        <v>295</v>
+        <v>298</v>
       </c>
       <c r="B36" s="56" t="n">
         <v>14450</v>
@@ -7865,7 +7887,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="1" t="s">
-        <v>296</v>
+        <v>299</v>
       </c>
       <c r="B37" s="56" t="n">
         <v>14870</v>
@@ -7873,7 +7895,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>297</v>
+        <v>300</v>
       </c>
       <c r="B38" s="56" t="n">
         <v>15290</v>
@@ -7881,7 +7903,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>298</v>
+        <v>301</v>
       </c>
       <c r="B39" s="56" t="n">
         <v>15710</v>
@@ -7889,7 +7911,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>299</v>
+        <v>302</v>
       </c>
       <c r="B40" s="56" t="n">
         <v>16130</v>
@@ -7897,7 +7919,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>300</v>
+        <v>303</v>
       </c>
       <c r="B41" s="56" t="n">
         <v>16540</v>
@@ -7905,7 +7927,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="B42" s="56" t="n">
         <v>16960</v>
@@ -7913,7 +7935,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="1" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="B43" s="56" t="n">
         <v>17380</v>
@@ -7921,7 +7943,7 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="1" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B44" s="56" t="n">
         <v>17800</v>
@@ -7929,7 +7951,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="1" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="B45" s="56" t="n">
         <v>18220</v>
@@ -7937,7 +7959,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="1" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B46" s="56" t="n">
         <v>18640</v>
@@ -7945,7 +7967,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="1" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="B47" s="56" t="n">
         <v>19060</v>
@@ -7953,7 +7975,7 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="1" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B48" s="56" t="n">
         <v>19470</v>
@@ -7961,7 +7983,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="1" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="B49" s="56" t="n">
         <v>19880</v>
@@ -7969,7 +7991,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="1" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B50" s="56" t="n">
         <v>20330</v>
@@ -7977,7 +7999,7 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="1" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="B51" s="56" t="n">
         <v>20900</v>
@@ -7985,7 +8007,7 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="1" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="B52" s="56" t="n">
         <v>21470</v>
@@ -7993,7 +8015,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="1" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="B53" s="56" t="n">
         <v>22040</v>
@@ -8001,7 +8023,7 @@
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="1" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="B54" s="56" t="n">
         <v>22430</v>
@@ -8009,7 +8031,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="1" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="B55" s="56" t="n">
         <v>22640</v>
@@ -8017,7 +8039,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="1" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="B56" s="56" t="n">
         <v>22860</v>
@@ -8025,7 +8047,7 @@
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="1" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
       <c r="B57" s="56" t="n">
         <v>23070</v>
@@ -8033,7 +8055,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="1" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B58" s="56" t="n">
         <v>23280</v>
@@ -8041,7 +8063,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="1" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="B59" s="56" t="n">
         <v>23600</v>
@@ -8049,7 +8071,7 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A60" s="1" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="B60" s="56" t="n">
         <v>24010</v>
@@ -8057,7 +8079,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A61" s="1" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="B61" s="56" t="n">
         <v>24430</v>
@@ -8065,7 +8087,7 @@
     </row>
     <row r="62" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A62" s="1" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
       <c r="B62" s="56" t="n">
         <v>24850</v>
@@ -8073,7 +8095,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A63" s="1" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="B63" s="56" t="n">
         <v>25260</v>
@@ -8081,7 +8103,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A64" s="1" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="B64" s="56" t="n">
         <v>25680</v>
@@ -8089,7 +8111,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A65" s="1" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="B65" s="56" t="n">
         <v>26090</v>
@@ -8097,7 +8119,7 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A66" s="1" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="B66" s="56" t="n">
         <v>26510</v>
@@ -8105,7 +8127,7 @@
     </row>
     <row r="67" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A67" s="1" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="B67" s="56" t="n">
         <v>26930</v>
@@ -8113,7 +8135,7 @@
     </row>
     <row r="68" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A68" s="1" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="B68" s="56" t="n">
         <v>27340</v>
@@ -8121,7 +8143,7 @@
     </row>
     <row r="69" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A69" s="1" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
       <c r="B69" s="56" t="n">
         <v>27730</v>
@@ -8129,7 +8151,7 @@
     </row>
     <row r="70" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A70" s="1" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="B70" s="56" t="n">
         <v>28080</v>
@@ -8137,7 +8159,7 @@
     </row>
     <row r="71" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A71" s="1" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
       <c r="B71" s="56" t="n">
         <v>28440</v>
@@ -8145,7 +8167,7 @@
     </row>
     <row r="72" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A72" s="1" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B72" s="56" t="n">
         <v>28800</v>
@@ -8153,7 +8175,7 @@
     </row>
     <row r="73" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A73" s="1" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B73" s="56" t="n">
         <v>29150</v>
@@ -8161,7 +8183,7 @@
     </row>
     <row r="74" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A74" s="1" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B74" s="56" t="n">
         <v>29570</v>
@@ -8169,7 +8191,7 @@
     </row>
     <row r="75" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A75" s="1" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
       <c r="B75" s="56" t="n">
         <v>30050</v>
@@ -8177,7 +8199,7 @@
     </row>
     <row r="76" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A76" s="1" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B76" s="56" t="n">
         <v>30530</v>
@@ -8185,7 +8207,7 @@
     </row>
     <row r="77" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A77" s="1" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
       <c r="B77" s="56" t="n">
         <v>31010</v>
@@ -8193,7 +8215,7 @@
     </row>
     <row r="78" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A78" s="1" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B78" s="56" t="n">
         <v>31490</v>
@@ -8201,7 +8223,7 @@
     </row>
     <row r="79" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A79" s="1" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
       <c r="B79" s="56" t="n">
         <v>31940</v>
@@ -8209,7 +8231,7 @@
     </row>
     <row r="80" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A80" s="1" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B80" s="56" t="n">
         <v>32360</v>
@@ -8217,7 +8239,7 @@
     </row>
     <row r="81" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A81" s="1" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
       <c r="B81" s="56" t="n">
         <v>32780</v>
@@ -8225,7 +8247,7 @@
     </row>
     <row r="82" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A82" s="1" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B82" s="56" t="n">
         <v>33210</v>
@@ -8233,7 +8255,7 @@
     </row>
     <row r="83" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A83" s="1" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
       <c r="B83" s="56" t="n">
         <v>33630</v>
@@ -8241,7 +8263,7 @@
     </row>
     <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A84" s="1" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
       <c r="B84" s="56" t="n">
         <v>34050</v>
@@ -8249,7 +8271,7 @@
     </row>
     <row r="85" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A85" s="1" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B85" s="56" t="n">
         <v>34470</v>
@@ -8257,7 +8279,7 @@
     </row>
     <row r="86" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A86" s="1" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="B86" s="56" t="n">
         <v>34900</v>
@@ -8265,7 +8287,7 @@
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A87" s="1" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B87" s="56" t="n">
         <v>35320</v>
@@ -8273,7 +8295,7 @@
     </row>
     <row r="88" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A88" s="1" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="B88" s="56" t="n">
         <v>35740</v>
@@ -8281,7 +8303,7 @@
     </row>
     <row r="89" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A89" s="1" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
       <c r="B89" s="56" t="n">
         <v>36160</v>
@@ -8289,7 +8311,7 @@
     </row>
     <row r="90" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="1" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B90" s="56" t="n">
         <v>36580</v>
@@ -8297,7 +8319,7 @@
     </row>
     <row r="91" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="1" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
       <c r="B91" s="56" t="n">
         <v>37000</v>
@@ -8305,7 +8327,7 @@
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A92" s="1" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="B92" s="56" t="n">
         <v>37410</v>
@@ -8313,7 +8335,7 @@
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A93" s="1" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
       <c r="B93" s="56" t="n">
         <v>37830</v>
@@ -8321,7 +8343,7 @@
     </row>
     <row r="94" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A94" s="1" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="B94" s="56" t="n">
         <v>38250</v>
@@ -8329,7 +8351,7 @@
     </row>
     <row r="95" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A95" s="1" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
       <c r="B95" s="56" t="n">
         <v>38670</v>
@@ -8337,7 +8359,7 @@
     </row>
     <row r="96" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A96" s="1" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="B96" s="56" t="n">
         <v>39080</v>
@@ -8345,7 +8367,7 @@
     </row>
     <row r="97" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A97" s="1" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
       <c r="B97" s="56" t="n">
         <v>39500</v>
@@ -8353,7 +8375,7 @@
     </row>
     <row r="98" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A98" s="1" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="B98" s="56" t="n">
         <v>39920</v>
@@ -8361,7 +8383,7 @@
     </row>
     <row r="99" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A99" s="1" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
       <c r="B99" s="56" t="n">
         <v>40340</v>
@@ -8369,7 +8391,7 @@
     </row>
     <row r="100" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A100" s="1" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="B100" s="56" t="n">
         <v>40750</v>
@@ -8377,7 +8399,7 @@
     </row>
     <row r="101" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A101" s="1" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
       <c r="B101" s="56" t="n">
         <v>41160</v>
@@ -8385,7 +8407,7 @@
     </row>
     <row r="102" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A102" s="1" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="B102" s="56" t="n">
         <v>41580</v>
@@ -8393,7 +8415,7 @@
     </row>
     <row r="103" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A103" s="1" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
       <c r="B103" s="56" t="n">
         <v>41990</v>
@@ -8401,7 +8423,7 @@
     </row>
     <row r="104" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A104" s="1" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="B104" s="56" t="n">
         <v>42410</v>
@@ -8409,7 +8431,7 @@
     </row>
     <row r="105" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A105" s="1" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
       <c r="B105" s="56" t="n">
         <v>42820</v>
@@ -8417,7 +8439,7 @@
     </row>
     <row r="106" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A106" s="1" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="B106" s="56" t="n">
         <v>43240</v>
@@ -8425,7 +8447,7 @@
     </row>
     <row r="107" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A107" s="1" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
       <c r="B107" s="56" t="n">
         <v>43660</v>
@@ -8433,7 +8455,7 @@
     </row>
     <row r="108" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A108" s="1" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="B108" s="56" t="n">
         <v>44070</v>
@@ -8441,7 +8463,7 @@
     </row>
     <row r="109" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A109" s="1" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
       <c r="B109" s="56" t="n">
         <v>44490</v>
@@ -8449,7 +8471,7 @@
     </row>
     <row r="110" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A110" s="1" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="B110" s="56" t="n">
         <v>44920</v>
@@ -8457,7 +8479,7 @@
     </row>
     <row r="111" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A111" s="1" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
       <c r="B111" s="56" t="n">
         <v>45340</v>
@@ -8465,7 +8487,7 @@
     </row>
     <row r="112" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A112" s="1" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B112" s="56" t="n">
         <v>45770</v>
@@ -8473,7 +8495,7 @@
     </row>
     <row r="113" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A113" s="1" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="B113" s="56" t="n">
         <v>46200</v>
@@ -8481,7 +8503,7 @@
     </row>
     <row r="114" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A114" s="1" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
       <c r="B114" s="56" t="n">
         <v>46620</v>
@@ -8489,7 +8511,7 @@
     </row>
     <row r="115" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A115" s="1" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="B115" s="56" t="n">
         <v>47030</v>
@@ -8497,7 +8519,7 @@
     </row>
     <row r="116" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A116" s="1" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
       <c r="B116" s="56" t="n">
         <v>47440</v>
@@ -8505,7 +8527,7 @@
     </row>
     <row r="117" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A117" s="1" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="B117" s="56" t="n">
         <v>47860</v>
@@ -8513,7 +8535,7 @@
     </row>
     <row r="118" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A118" s="1" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="B118" s="56" t="n">
         <v>48270</v>
@@ -8521,7 +8543,7 @@
     </row>
     <row r="119" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A119" s="1" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
       <c r="B119" s="56" t="n">
         <v>48690</v>
@@ -8529,7 +8551,7 @@
     </row>
     <row r="120" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A120" s="1" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="B120" s="56" t="n">
         <v>49110</v>
@@ -8537,7 +8559,7 @@
     </row>
     <row r="121" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A121" s="1" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
       <c r="B121" s="56" t="n">
         <v>49540</v>
@@ -8545,7 +8567,7 @@
     </row>
     <row r="122" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A122" s="1" t="s">
-        <v>381</v>
+        <v>384</v>
       </c>
       <c r="B122" s="56" t="n">
         <v>49960</v>
@@ -8553,7 +8575,7 @@
     </row>
     <row r="123" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A123" s="1" t="s">
-        <v>382</v>
+        <v>385</v>
       </c>
       <c r="B123" s="56" t="n">
         <v>50380</v>
@@ -8583,7 +8605,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>383</v>
+        <v>386</v>
       </c>
       <c r="C1" s="69" t="n">
         <v>2026</v>
@@ -8591,10 +8613,10 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="70" t="s">
-        <v>384</v>
+        <v>387</v>
       </c>
       <c r="B2" s="70" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="C2" s="71" t="n">
         <v>2885</v>
@@ -8602,7 +8624,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="70" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="C3" s="71" t="n">
         <v>3303</v>
@@ -8610,7 +8632,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="70" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="C4" s="71" t="n">
         <v>3756</v>
@@ -8618,7 +8640,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="70" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="C5" s="71" t="n">
         <v>4314</v>
@@ -8626,7 +8648,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B6" s="70" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="C6" s="71" t="n">
         <v>5315</v>
@@ -8634,7 +8656,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B7" s="70" t="s">
-        <v>390</v>
+        <v>393</v>
       </c>
       <c r="C7" s="71" t="n">
         <v>6275</v>
@@ -8642,7 +8664,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B8" s="70" t="s">
-        <v>391</v>
+        <v>394</v>
       </c>
       <c r="C8" s="71" t="n">
         <v>7306</v>
@@ -8650,7 +8672,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B9" s="70" t="s">
-        <v>392</v>
+        <v>395</v>
       </c>
       <c r="C9" s="1" t="n">
         <v>8308</v>
@@ -8658,7 +8680,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B10" s="70" t="s">
-        <v>393</v>
+        <v>396</v>
       </c>
       <c r="C10" s="1" t="n">
         <v>9278</v>
@@ -8666,7 +8688,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B11" s="70" t="s">
-        <v>394</v>
+        <v>397</v>
       </c>
       <c r="C11" s="1" t="n">
         <v>10392</v>
@@ -8674,7 +8696,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="70" t="s">
-        <v>395</v>
+        <v>398</v>
       </c>
       <c r="C12" s="1" t="n">
         <v>11228</v>
@@ -8682,12 +8704,12 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B13" s="70" t="s">
-        <v>396</v>
+        <v>399</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B14" s="70" t="s">
-        <v>397</v>
+        <v>400</v>
       </c>
       <c r="C14" s="1" t="n">
         <v>18</v>
@@ -8717,12 +8739,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>398</v>
+        <v>401</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="72" t="s">
-        <v>399</v>
+        <v>402</v>
       </c>
       <c r="B2" s="73" t="n">
         <v>2026</v>
@@ -8730,7 +8752,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="72" t="s">
-        <v>400</v>
+        <v>403</v>
       </c>
       <c r="B3" s="70" t="n">
         <v>1430</v>
@@ -8738,7 +8760,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="72" t="s">
-        <v>401</v>
+        <v>404</v>
       </c>
       <c r="B4" s="70" t="n">
         <v>1640</v>
@@ -8746,7 +8768,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="72" t="s">
-        <v>402</v>
+        <v>405</v>
       </c>
       <c r="B5" s="70" t="n">
         <v>1880</v>
@@ -8754,7 +8776,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="72" t="s">
-        <v>403</v>
+        <v>406</v>
       </c>
       <c r="B6" s="70" t="n">
         <v>2100</v>
@@ -8762,7 +8784,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="72" t="s">
-        <v>404</v>
+        <v>407</v>
       </c>
       <c r="B7" s="70" t="n">
         <v>2300</v>
@@ -8770,7 +8792,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="70" t="s">
-        <v>405</v>
+        <v>408</v>
       </c>
       <c r="B8" s="70" t="n">
         <v>2600</v>
@@ -8778,10 +8800,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="72" t="s">
-        <v>406</v>
+        <v>409</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>407</v>
+        <v>410</v>
       </c>
       <c r="C10" s="74" t="n">
         <v>790</v>
@@ -8811,7 +8833,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="75" t="s">
-        <v>408</v>
+        <v>411</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8821,7 +8843,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="76" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>7410</v>
@@ -8829,7 +8851,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>10550</v>
@@ -8837,7 +8859,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>13830</v>
@@ -8845,7 +8867,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>17510</v>
@@ -8875,12 +8897,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>409</v>
+        <v>412</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="77" t="s">
-        <v>385</v>
+        <v>388</v>
       </c>
       <c r="B2" s="1" t="n">
         <v>2580</v>
@@ -8888,7 +8910,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="78" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>3100</v>
@@ -8896,7 +8918,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="78" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3600</v>
@@ -8904,7 +8926,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="78" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>4150</v>
@@ -8912,7 +8934,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="78" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>4640</v>
@@ -8920,7 +8942,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="78" t="s">
-        <v>410</v>
+        <v>413</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>32</v>
@@ -8950,7 +8972,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>411</v>
+        <v>414</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8960,7 +8982,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="s">
-        <v>412</v>
+        <v>415</v>
       </c>
       <c r="B3" s="1" t="n">
         <v>2580</v>
@@ -8968,7 +8990,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="s">
-        <v>386</v>
+        <v>389</v>
       </c>
       <c r="B4" s="1" t="n">
         <v>3090</v>
@@ -8976,7 +8998,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="s">
-        <v>387</v>
+        <v>390</v>
       </c>
       <c r="B5" s="1" t="n">
         <v>3610</v>
@@ -8984,7 +9006,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="s">
-        <v>388</v>
+        <v>391</v>
       </c>
       <c r="B6" s="1" t="n">
         <v>4130</v>
@@ -8992,7 +9014,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="s">
-        <v>389</v>
+        <v>392</v>
       </c>
       <c r="B7" s="1" t="n">
         <v>4640</v>
@@ -9000,7 +9022,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="70" t="s">
-        <v>413</v>
+        <v>416</v>
       </c>
     </row>
   </sheetData>

</xml_diff>